<commit_message>
data: start Tang Liangjing volume 3 extraction
</commit_message>
<xml_diff>
--- a/00-项目总览/唐长安城知识图谱_项目进度看板.xlsx
+++ b/00-项目总览/唐长安城知识图谱_项目进度看板.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日看板" sheetId="1" r:id="R9daafb6472ed41e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作清单" sheetId="2" r:id="R3a42c3f39b6e4ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="里程碑" sheetId="3" r:id="R1cc9542668834a03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="4" r:id="Rc0cf334afc864143"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日看板" sheetId="1" r:id="R446bd1c839944d24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作清单" sheetId="2" r:id="R36710fc17ea9411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="里程碑" sheetId="3" r:id="R95b4a19c0cfd4c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="4" r:id="Rcb0523960099494a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1656,7 +1656,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R26db6e3eb3ad448a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R69de101977074714"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1959,7 +1959,7 @@
     <x:row r="6" ht="32" customHeight="1">
       <x:c r="A6" s="449" t="n">
         <x:f>COUNTA('工作清单'!$A$4:$A$200)</x:f>
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B6" s="449"/>
       <x:c r="C6" s="449"/>
@@ -1971,13 +1971,13 @@
       <x:c r="F6" s="449"/>
       <x:c r="G6" s="450" t="n">
         <x:f>COUNTIF('工作清单'!$E$4:$E$200,"进行中")</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H6" s="450"/>
       <x:c r="I6" s="450"/>
       <x:c r="J6" s="451" t="n">
         <x:f>IFERROR(D6/A6,0)</x:f>
-        <x:v>0.5625</x:v>
+        <x:v>0.5538461538461539</x:v>
       </x:c>
       <x:c r="K6" s="347"/>
       <x:c r="L6" s="347"/>
@@ -2036,9 +2036,9 @@
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="453" t="str">
-        <x:v>《唐两京城坊考》卷一、卷二已联合导入18081平台
-联合包：765个去重实体、1128条去重关系、72个史料片段
-平台总量：812个实体、1205条关系、104个史料片段；已验收</x:v>
+        <x:v>当前阶段：成员A开始《唐两京城坊考》卷三
+首批完成翊善—光宅、永昌—来庭两组分坊沿革
+卷三当前：4个完整史料片段、2个稳定坊、20处建筑设施、23条关系；已自主审核并通过结构校验</x:v>
       </x:c>
       <x:c r="B10" s="454"/>
       <x:c r="C10" s="454"/>
@@ -2110,7 +2110,9 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="459" t="str">
-        <x:v>下一步：在网页抽查卷二坊、建筑和跨卷双证据关系，然后开始卷三。</x:v>
+        <x:v>1. 继续东第三街：永兴坊起，按原文顺序逐坊录入。
+2. 分坊沿革继续采用稳定坊编号＋历史名称证据的做法。
+3. 每批同步填写专题表、实体表、关系表并检查孤立实体与重复边。</x:v>
       </x:c>
       <x:c r="B15" s="460"/>
       <x:c r="C15" s="460"/>
@@ -2260,7 +2262,7 @@
     <x:mergeCell ref="A20:L22"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R272a654ae9db43e6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3d600b45bab45ad"/>
 </x:worksheet>
 </file>
 
@@ -4576,6 +4578,40 @@
       </x:c>
       <x:c r="L67" s="446" t="str">
         <x:v>卷二累计13片段、74实体、98关系；东第一列9坊及49处设施已录；2项名称待扫描版复核</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>S7-09</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>阶段七：全量提取</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>启动《唐两京城坊考》卷三并完成首批分坊沿革</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>成员A / Codex</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>进行中</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>2026-08-16</x:v>
+      </x:c>
+      <x:c r="H68"/>
+      <x:c r="I68"/>
+      <x:c r="J68" t="str">
+        <x:v>继续东第三街永兴坊以后条目</x:v>
+      </x:c>
+      <x:c r="K68" t="str">
+        <x:v>BATCH-0202工作簿 / 协作登记表</x:v>
+      </x:c>
+      <x:c r="L68" t="str">
+        <x:v>4片段、20设施、23关系；复用TC-FANG-0023/0024</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4895,7 +4931,7 @@
       <x:c r="E4" s="207" t="str">
         <x:v>复制并建立新平台仓库</x:v>
       </x:c>
-      <x:c r="F4" s="207" t="str"/>
+      <x:c r="F4" s="207"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="207" t="str">
@@ -4933,7 +4969,7 @@
       <x:c r="E6" s="207" t="str">
         <x:v>组织六张表字段联合评审</x:v>
       </x:c>
-      <x:c r="F6" s="207" t="str"/>
+      <x:c r="F6" s="207"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="207" t="str">
@@ -5893,6 +5929,26 @@
       </x:c>
       <x:c r="F54" s="446" t="str">
         <x:v>已移除包内v3.1 Skill和旧v1手册；5个Excel公式错误扫描均为0，Word三页版式检查通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>2026-08-16</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>成员A / Codex</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>启动卷三并完成翊善—光宅、永昌—来庭首批提取</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>卷三工作簿 / 协作登记表 / 项目看板</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>继续东第三街后续各坊</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>四段原文独立保留；实体层复用两个稳定坊编号；新增20处设施</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
data: complete Tang Liangjing volume 3 extraction
</commit_message>
<xml_diff>
--- a/00-项目总览/唐长安城知识图谱_项目进度看板.xlsx
+++ b/00-项目总览/唐长安城知识图谱_项目进度看板.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日看板" sheetId="1" r:id="R446bd1c839944d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作清单" sheetId="2" r:id="R36710fc17ea9411d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="里程碑" sheetId="3" r:id="R95b4a19c0cfd4c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="4" r:id="Rcb0523960099494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日看板" sheetId="1" r:id="R034e1f087500450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作清单" sheetId="2" r:id="R697e5460a98341b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="里程碑" sheetId="3" r:id="Rc085725758e04211"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="4" r:id="Rd9794bbe0c954033"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -86,8 +86,14 @@
       <x:color rgb="FF333333"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -189,6 +195,16 @@
         <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F3E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F3E8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="13">
     <x:border/>
@@ -280,7 +296,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="468">
+  <x:cellXfs count="498">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1391,6 +1407,96 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1656,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R69de101977074714"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R432aaa9fcf1a4272"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1965,19 +2071,19 @@
       <x:c r="C6" s="449"/>
       <x:c r="D6" s="449" t="n">
         <x:f>COUNTIF('工作清单'!$E$4:$E$200,"已完成")</x:f>
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E6" s="449"/>
       <x:c r="F6" s="449"/>
       <x:c r="G6" s="450" t="n">
         <x:f>COUNTIF('工作清单'!$E$4:$E$200,"进行中")</x:f>
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H6" s="450"/>
       <x:c r="I6" s="450"/>
       <x:c r="J6" s="451" t="n">
         <x:f>IFERROR(D6/A6,0)</x:f>
-        <x:v>0.5538461538461539</x:v>
+        <x:v>0.5692307692307692</x:v>
       </x:c>
       <x:c r="K6" s="347"/>
       <x:c r="L6" s="347"/>
@@ -2034,49 +2140,49 @@
       <x:c r="N9"/>
       <x:c r="O9"/>
     </x:row>
-    <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="453" t="str">
-        <x:v>当前阶段：成员A开始《唐两京城坊考》卷三
-首批完成翊善—光宅、永昌—来庭两组分坊沿革
-卷三当前：4个完整史料片段、2个稳定坊、20处建筑设施、23条关系；已自主审核并通过结构校验</x:v>
-      </x:c>
-      <x:c r="B10" s="454"/>
-      <x:c r="C10" s="454"/>
-      <x:c r="D10" s="454"/>
-      <x:c r="E10" s="454"/>
-      <x:c r="F10" s="454"/>
-      <x:c r="G10" s="454"/>
-      <x:c r="H10" s="454"/>
-      <x:c r="I10" s="454"/>
-      <x:c r="J10" s="454"/>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="492" t="str">
+        <x:v>当前阶段：《唐两京城坊考》卷三已完成
+全卷40个完整史料片段，35个坊，408处正文直述建筑/设施，451个实体，448条关系
+东市、曲江、芙蓉园已作为专题区域录入；普通事实已AI自主审核，下一步为平台联合验收</x:v>
+      </x:c>
+      <x:c r="B10" s="493"/>
+      <x:c r="C10" s="493"/>
+      <x:c r="D10" s="493"/>
+      <x:c r="E10" s="493"/>
+      <x:c r="F10" s="493"/>
+      <x:c r="G10" s="493"/>
+      <x:c r="H10" s="493"/>
+      <x:c r="I10" s="493"/>
+      <x:c r="J10" s="493"/>
       <x:c r="K10" s="371"/>
       <x:c r="L10" s="372"/>
     </x:row>
-    <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="455"/>
-      <x:c r="B11" s="456"/>
-      <x:c r="C11" s="456"/>
-      <x:c r="D11" s="456"/>
-      <x:c r="E11" s="456"/>
-      <x:c r="F11" s="456"/>
-      <x:c r="G11" s="456"/>
-      <x:c r="H11" s="456"/>
-      <x:c r="I11" s="456"/>
-      <x:c r="J11" s="456"/>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="494"/>
+      <x:c r="B11" s="495"/>
+      <x:c r="C11" s="495"/>
+      <x:c r="D11" s="495"/>
+      <x:c r="E11" s="495"/>
+      <x:c r="F11" s="495"/>
+      <x:c r="G11" s="495"/>
+      <x:c r="H11" s="495"/>
+      <x:c r="I11" s="495"/>
+      <x:c r="J11" s="495"/>
       <x:c r="K11" s="374"/>
       <x:c r="L11" s="375"/>
     </x:row>
-    <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="457"/>
-      <x:c r="B12" s="458"/>
-      <x:c r="C12" s="458"/>
-      <x:c r="D12" s="458"/>
-      <x:c r="E12" s="458"/>
-      <x:c r="F12" s="458"/>
-      <x:c r="G12" s="458"/>
-      <x:c r="H12" s="458"/>
-      <x:c r="I12" s="458"/>
-      <x:c r="J12" s="458"/>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="496"/>
+      <x:c r="B12" s="497"/>
+      <x:c r="C12" s="497"/>
+      <x:c r="D12" s="497"/>
+      <x:c r="E12" s="497"/>
+      <x:c r="F12" s="497"/>
+      <x:c r="G12" s="497"/>
+      <x:c r="H12" s="497"/>
+      <x:c r="I12" s="497"/>
+      <x:c r="J12" s="497"/>
       <x:c r="K12" s="377"/>
       <x:c r="L12" s="378"/>
     </x:row>
@@ -2108,49 +2214,49 @@
       <x:c r="K14" s="351"/>
       <x:c r="L14" s="351"/>
     </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="459" t="str">
-        <x:v>1. 继续东第三街：永兴坊起，按原文顺序逐坊录入。
-2. 分坊沿革继续采用稳定坊编号＋历史名称证据的做法。
-3. 每批同步填写专题表、实体表、关系表并检查孤立实体与重复边。</x:v>
-      </x:c>
-      <x:c r="B15" s="460"/>
-      <x:c r="C15" s="460"/>
-      <x:c r="D15" s="460"/>
-      <x:c r="E15" s="460"/>
-      <x:c r="F15" s="460"/>
-      <x:c r="G15" s="460"/>
-      <x:c r="H15" s="460"/>
-      <x:c r="I15" s="460"/>
-      <x:c r="J15" s="460"/>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="492" t="str">
+        <x:v>1. 将卷三与卷一、卷二按稳定ID联合导入测试平台。
+2. 网页抽查东第三、第四、第五街及东市、曲江、芙蓉园。
+3. 对扫描页码和电子文本疑似讹字保留后续专项复核入口。</x:v>
+      </x:c>
+      <x:c r="B15" s="493"/>
+      <x:c r="C15" s="493"/>
+      <x:c r="D15" s="493"/>
+      <x:c r="E15" s="493"/>
+      <x:c r="F15" s="493"/>
+      <x:c r="G15" s="493"/>
+      <x:c r="H15" s="493"/>
+      <x:c r="I15" s="493"/>
+      <x:c r="J15" s="493"/>
       <x:c r="K15" s="398"/>
       <x:c r="L15" s="399"/>
     </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="461"/>
-      <x:c r="B16" s="462"/>
-      <x:c r="C16" s="462"/>
-      <x:c r="D16" s="462"/>
-      <x:c r="E16" s="462"/>
-      <x:c r="F16" s="462"/>
-      <x:c r="G16" s="462"/>
-      <x:c r="H16" s="462"/>
-      <x:c r="I16" s="462"/>
-      <x:c r="J16" s="462"/>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="494"/>
+      <x:c r="B16" s="495"/>
+      <x:c r="C16" s="495"/>
+      <x:c r="D16" s="495"/>
+      <x:c r="E16" s="495"/>
+      <x:c r="F16" s="495"/>
+      <x:c r="G16" s="495"/>
+      <x:c r="H16" s="495"/>
+      <x:c r="I16" s="495"/>
+      <x:c r="J16" s="495"/>
       <x:c r="K16" s="401"/>
       <x:c r="L16" s="402"/>
     </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="463"/>
-      <x:c r="B17" s="464"/>
-      <x:c r="C17" s="464"/>
-      <x:c r="D17" s="464"/>
-      <x:c r="E17" s="464"/>
-      <x:c r="F17" s="464"/>
-      <x:c r="G17" s="464"/>
-      <x:c r="H17" s="464"/>
-      <x:c r="I17" s="464"/>
-      <x:c r="J17" s="464"/>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="496"/>
+      <x:c r="B17" s="497"/>
+      <x:c r="C17" s="497"/>
+      <x:c r="D17" s="497"/>
+      <x:c r="E17" s="497"/>
+      <x:c r="F17" s="497"/>
+      <x:c r="G17" s="497"/>
+      <x:c r="H17" s="497"/>
+      <x:c r="I17" s="497"/>
+      <x:c r="J17" s="497"/>
       <x:c r="K17" s="404"/>
       <x:c r="L17" s="405"/>
     </x:row>
@@ -2255,14 +2361,14 @@
     <x:mergeCell ref="G6:I6"/>
     <x:mergeCell ref="J6:L6"/>
     <x:mergeCell ref="A9:L9"/>
-    <x:mergeCell ref="A10:L12"/>
     <x:mergeCell ref="A14:L14"/>
-    <x:mergeCell ref="A15:L17"/>
     <x:mergeCell ref="A19:L19"/>
     <x:mergeCell ref="A20:L22"/>
+    <x:mergeCell ref="A10:J12"/>
+    <x:mergeCell ref="A15:J17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3d600b45bab45ad"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R206551128a224f8e"/>
 </x:worksheet>
 </file>
 
@@ -4594,7 +4700,7 @@
         <x:v>成员A / Codex</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>进行中</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="F68" t="str">
         <x:v>P0</x:v>
@@ -4605,13 +4711,13 @@
       <x:c r="H68"/>
       <x:c r="I68"/>
       <x:c r="J68" t="str">
-        <x:v>继续东第三街永兴坊以后条目</x:v>
+        <x:v>联合导入卷一至卷三并网页验收</x:v>
       </x:c>
       <x:c r="K68" t="str">
         <x:v>BATCH-0202工作簿 / 协作登记表</x:v>
       </x:c>
       <x:c r="L68" t="str">
-        <x:v>4片段、20设施、23关系；复用TC-FANG-0023/0024</x:v>
+        <x:v>卷三40片段、35坊、408设施、451实体、448关系；结构校验通过</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5951,6 +6057,26 @@
         <x:v>四段原文独立保留；实体层复用两个稳定坊编号；新增20处设施</x:v>
       </x:c>
     </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>2026-08-16</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>成员A / Codex</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>完成《唐两京城坊考》卷三全卷提取、自主审核与图谱转换</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>卷三工作簿 / 协作登记表 / 项目看板</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>卷一至卷三联合导入与网页验收</x:v>
+      </x:c>
+      <x:c r="F56" t="str">
+        <x:v>完成道路编号纠错；东市、曲江、芙蓉园新增Area实体；建筑编号用至TC-BUILDING-2943</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>